<commit_message>
docs: docs/leaderboard.xlsx 실험 기록 업데이트
</commit_message>
<xml_diff>
--- a/docs/leaderboard.xlsx
+++ b/docs/leaderboard.xlsx
@@ -69,7 +69,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -107,25 +107,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00B0B8D0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00B0B8D0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00B0B8D0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00B0B8D0"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -156,24 +142,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -540,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S18"/>
+  <dimension ref="A1:S38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -660,7 +628,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -718,7 +686,7 @@
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>N</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr">
@@ -738,7 +706,7 @@
       </c>
       <c r="S2" s="4" t="inlineStr">
         <is>
-          <t>클래스 불균형 2.87:1. is_unbalance=True 적용. OOF 0.73887 기준점 확보</t>
+          <t xml:space="preserve">클래스 불균형 2.87:1. is_unbalance=True 적용. OOF 0.73887 기준점 확보, 여기까지 preprocessing.py 전처리에 Data Leakage 있었는데, </t>
         </is>
       </c>
     </row>
@@ -1707,326 +1675,1958 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>2026-04-25</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>EXP-017</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>조여진</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>LGB+PseudoLabel</t>
         </is>
       </c>
-      <c r="E15" s="12" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>LGB + pseudo_label(th=0.85/0.1) | pseudo=13,784샘플 | Round1=0.73864 → Round2=0.73885</t>
         </is>
       </c>
-      <c r="F15" s="13" t="n">
+      <c r="F15" s="8" t="n">
         <v>0.51642</v>
       </c>
-      <c r="G15" s="13" t="n">
+      <c r="G15" s="8" t="n">
         <v>0.81007</v>
       </c>
-      <c r="H15" s="13" t="n">
+      <c r="H15" s="8" t="n">
         <v>0.37902</v>
       </c>
-      <c r="I15" s="13" t="n">
+      <c r="I15" s="8" t="n">
         <v>0.60805</v>
       </c>
-      <c r="J15" s="13" t="n">
+      <c r="J15" s="8" t="n">
         <v>0.73885</v>
       </c>
-      <c r="K15" s="11" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>Stratified 5-Fold</t>
         </is>
       </c>
-      <c r="L15" s="12" t="inlineStr">
+      <c r="L15" s="7" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="M15" s="11" t="n">
+      <c r="M15" s="6" t="n">
         <v>85</v>
       </c>
-      <c r="N15" s="12" t="inlineStr">
+      <c r="N15" s="7" t="inlineStr">
         <is>
           <t>is_unbalance=True</t>
         </is>
       </c>
-      <c r="O15" s="11" t="inlineStr">
+      <c r="O15" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="P15" s="13" t="n"/>
-      <c r="Q15" s="12" t="inlineStr">
+      <c r="P15" s="8" t="n"/>
+      <c r="Q15" s="7" t="inlineStr">
         <is>
           <t>notebooks/13_pseudo_label_yjcho.ipynb</t>
         </is>
       </c>
-      <c r="R15" s="12" t="inlineStr">
+      <c r="R15" s="7" t="inlineStr">
         <is>
           <t>Pseudo-labeling 2-Round. 임계값 0.85/0.1, pseudo 13,784샘플 추가</t>
         </is>
       </c>
-      <c r="S15" s="12" t="inlineStr">
-        <is>
-          <t>Round1→2: +0.00021 | pos=0 neg=13,784</t>
+      <c r="S15" s="7" t="inlineStr">
+        <is>
+          <t>해커톤 규칙 위반에 해당할 가능성 있음</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>2026-04-25</t>
         </is>
       </c>
-      <c r="B16" s="14" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>EXP-018</t>
         </is>
       </c>
-      <c r="C16" s="14" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>조여진</t>
         </is>
       </c>
-      <c r="D16" s="15" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Ensemble-v3(LGB+CAT+XGB+RF)</t>
         </is>
       </c>
-      <c r="E16" s="15" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>LGB+CAT(EXP-011)+XGB(EXP-012)+RF(n=1000) | best=Optuna Weights | LGB=0.079 CAT=0.274 XGB=0.631 RF=0.015</t>
         </is>
       </c>
-      <c r="F16" s="16" t="n">
+      <c r="F16" s="5" t="n">
         <v>0.5176500000000001</v>
       </c>
-      <c r="G16" s="16" t="n">
+      <c r="G16" s="5" t="n">
         <v>0.7815299999999999</v>
       </c>
-      <c r="H16" s="16" t="n">
+      <c r="H16" s="5" t="n">
         <v>0.38699</v>
       </c>
-      <c r="I16" s="16" t="n">
+      <c r="I16" s="5" t="n">
         <v>0.62373</v>
       </c>
-      <c r="J16" s="16" t="n">
+      <c r="J16" s="5" t="n">
         <v>0.74063</v>
       </c>
-      <c r="K16" s="14" t="inlineStr">
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>Stratified 5-Fold</t>
         </is>
       </c>
-      <c r="L16" s="15" t="inlineStr">
+      <c r="L16" s="4" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="M16" s="3" t="n">
         <v>85</v>
       </c>
-      <c r="N16" s="15" t="inlineStr">
+      <c r="N16" s="4" t="inlineStr">
         <is>
           <t>is_unbalance / Balanced / scale_pos_weight / class_weight=balanced</t>
         </is>
       </c>
-      <c r="O16" s="14" t="inlineStr">
+      <c r="O16" s="3" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="P16" s="16" t="n"/>
-      <c r="Q16" s="15" t="inlineStr">
+      <c r="P16" s="5" t="n"/>
+      <c r="Q16" s="4" t="inlineStr">
         <is>
           <t>notebooks/14_ensemble_rf_yjcho.ipynb</t>
         </is>
       </c>
-      <c r="R16" s="15" t="inlineStr">
+      <c r="R16" s="4" t="inlineStr">
         <is>
           <t>RF 추가 4모델 앙상블. best=Optuna Weights</t>
         </is>
       </c>
-      <c r="S16" s="15" t="inlineStr">
+      <c r="S16" s="4" t="inlineStr">
         <is>
           <t>EXP-015 대비 +0.00017 | RF 단독 AUC=0.73485 | RF 가중치=0.015</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>2026-04-25</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>EXP-019</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>조여진</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>LightGBM(Optuna)</t>
         </is>
       </c>
-      <c r="E17" s="12" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>learning_rate=0.03543, num_leaves=266, max_depth=5, min_child_samples=166, feature_fraction=0.5346, bagging_fraction=0.7122, lambda_l1=9.901, lambda_l2=2.214, min_gain_to_split=0.1142</t>
         </is>
       </c>
-      <c r="F17" s="13" t="n">
+      <c r="F17" s="8" t="n">
         <v>0.51722</v>
       </c>
-      <c r="G17" s="13" t="n">
+      <c r="G17" s="8" t="n">
         <v>0.78172</v>
       </c>
-      <c r="H17" s="13" t="n">
+      <c r="H17" s="8" t="n">
         <v>0.38646</v>
       </c>
-      <c r="I17" s="13" t="n">
+      <c r="I17" s="8" t="n">
         <v>0.62298</v>
       </c>
-      <c r="J17" s="13" t="n">
+      <c r="J17" s="8" t="n">
         <v>0.74047</v>
       </c>
-      <c r="K17" s="11" t="inlineStr">
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>Stratified 5-Fold</t>
         </is>
       </c>
-      <c r="L17" s="12" t="inlineStr">
+      <c r="L17" s="7" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="M17" s="11" t="n">
+      <c r="M17" s="6" t="n">
         <v>85</v>
       </c>
-      <c r="N17" s="12" t="inlineStr">
+      <c r="N17" s="7" t="inlineStr">
         <is>
           <t>is_unbalance=True</t>
         </is>
       </c>
-      <c r="O17" s="11" t="inlineStr">
+      <c r="O17" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="P17" s="13" t="n"/>
-      <c r="Q17" s="12" t="inlineStr">
+      <c r="P17" s="8" t="n"/>
+      <c r="Q17" s="7" t="inlineStr">
         <is>
           <t>notebooks/15_hparam_lgb_yjcho.ipynb</t>
         </is>
       </c>
-      <c r="R17" s="12" t="inlineStr">
+      <c r="R17" s="7" t="inlineStr">
         <is>
           <t>LGB Optuna 50trials. 기존 고정 파라미터 대비 +0.00183</t>
         </is>
       </c>
-      <c r="S17" s="12" t="inlineStr">
+      <c r="S17" s="7" t="inlineStr">
         <is>
           <t>CAT 대비 +0.00044 / XGB 대비 +0.00031</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>2026-04-25</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>EXP-020</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>조여진</t>
         </is>
       </c>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Ensemble-v4(LGB+CAT+XGB, all-tuned)</t>
         </is>
       </c>
-      <c r="E18" s="15" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>LGB(EXP-019)+CAT(EXP-011)+XGB(EXP-012) | best=Rank Average | LGB=0.347 CAT=0.240 XGB=0.413</t>
         </is>
       </c>
-      <c r="F18" s="16" t="n">
+      <c r="F18" s="5" t="n">
         <v>0.41062</v>
       </c>
-      <c r="G18" s="16" t="n">
+      <c r="G18" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H18" s="16" t="n">
+      <c r="H18" s="5" t="n">
         <v>0.25835</v>
       </c>
-      <c r="I18" s="16" t="n">
+      <c r="I18" s="5" t="n">
         <v>0.25835</v>
       </c>
-      <c r="J18" s="16" t="n">
+      <c r="J18" s="5" t="n">
         <v>0.74068</v>
       </c>
-      <c r="K18" s="14" t="inlineStr">
+      <c r="K18" s="3" t="inlineStr">
         <is>
           <t>Stratified 5-Fold</t>
         </is>
       </c>
-      <c r="L18" s="15" t="inlineStr">
+      <c r="L18" s="4" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="M18" s="14" t="n">
+      <c r="M18" s="3" t="n">
         <v>85</v>
       </c>
-      <c r="N18" s="15" t="inlineStr">
+      <c r="N18" s="4" t="inlineStr">
         <is>
           <t>is_unbalance / Balanced / scale_pos_weight</t>
         </is>
       </c>
-      <c r="O18" s="14" t="inlineStr">
+      <c r="O18" s="3" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="P18" s="16" t="n"/>
-      <c r="Q18" s="15" t="inlineStr">
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 0.7421708074</t>
+        </is>
+      </c>
+      <c r="Q18" s="4" t="inlineStr">
         <is>
           <t>notebooks/16_ensemble_v4_yjcho.ipynb</t>
         </is>
       </c>
-      <c r="R18" s="15" t="inlineStr">
+      <c r="R18" s="4" t="inlineStr">
         <is>
           <t>3모델 전부 Optuna 튜닝. best=Rank Average</t>
         </is>
       </c>
-      <c r="S18" s="15" t="inlineStr">
+      <c r="S18" s="4" t="inlineStr">
         <is>
           <t>EXP-015 대비 +0.00022 | LGB=0.74047 CAT=0.74015 XGB=0.74051</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>EXP-021</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Ensemble(FE-v2)</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>FE-v2(+4피처) | LGB(EXP-019)+CAT(EXP-011)+XGB(EXP-012) | best=Rank Average</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>0.41062</v>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>0.25835</v>
+      </c>
+      <c r="I19" s="8" t="n">
+        <v>0.25835</v>
+      </c>
+      <c r="J19" s="8" t="n">
+        <v>0.74048</v>
+      </c>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="M19" s="6" t="n">
+        <v>89</v>
+      </c>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O19" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P19" s="8" t="n"/>
+      <c r="Q19" s="7" t="inlineStr">
+        <is>
+          <t>notebooks/17_fe_v2_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R19" s="7" t="inlineStr">
+        <is>
+          <t>FE v2: 임신_성공률 / 시술_실패_횟수 / 최적_난자수 / 나이_이식배아수 추가</t>
+        </is>
+      </c>
+      <c r="S19" s="7" t="inlineStr">
+        <is>
+          <t>EXP-020 대비 +0.00002 | 피처 수 89개</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>EXP-022</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Stacking-v2(LGB+CAT+XGB→LGB)</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Base:LGB(EXP-019)+CAT(EXP-011)+XGB(EXP-012) | Meta:LGB(num_leaves=8)</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>0.51733</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>0.77274</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>0.38881</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>0.62747</v>
+      </c>
+      <c r="J20" s="5" t="n">
+        <v>0.73999</v>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="n"/>
+      <c r="Q20" s="4" t="inlineStr">
+        <is>
+          <t>notebooks/18_stacking_lgb_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R20" s="4" t="inlineStr">
+        <is>
+          <t>Stacking v2: 메타 러너 LogisticRegression → LightGBM 교체</t>
+        </is>
+      </c>
+      <c r="S20" s="4" t="inlineStr">
+        <is>
+          <t>EXP-020 대비 -0.00047 | base LGB=0.74047 CAT=0.74015 XGB=0.74051</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>EXP-023</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Ensemble(FE-v2+TE)</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>FE-v2 + TE(9cols,alpha=10) | LGB(EXP-019)+CAT(EXP-011)+XGB(EXP-012) | best=Rank Average</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>0.41062</v>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>0.25835</v>
+      </c>
+      <c r="I21" s="8" t="n">
+        <v>0.25835</v>
+      </c>
+      <c r="J21" s="8" t="n">
+        <v>0.74063</v>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t>v2+TE</t>
+        </is>
+      </c>
+      <c r="M21" s="6" t="n">
+        <v>98</v>
+      </c>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O21" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P21" s="8" t="n"/>
+      <c r="Q21" s="7" t="inlineStr">
+        <is>
+          <t>notebooks/19_target_encoding_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R21" s="7" t="inlineStr">
+        <is>
+          <t>Target Encoding 9개 컬럼 추가 (명목형6+순서형3), KFold OOF 방식</t>
+        </is>
+      </c>
+      <c r="S21" s="7" t="inlineStr">
+        <is>
+          <t>EXP-021 대비 +0.00015 | base LGB=0.74041 CAT=0.74022 XGB=0.74035 | 피처 수 98</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>EXP-024</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Ensemble(FE-v2+TE+ITE)</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>FE-v2 + TE(9cols) + ITE(6pairs) | LGB(EXP-019)+CAT(EXP-011)+XGB(EXP-012) | best=Rank Average</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>0.41062</v>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>0.25835</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>0.25835</v>
+      </c>
+      <c r="J22" s="5" t="n">
+        <v>0.74061</v>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>v2+TE+ITE</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="n">
+        <v>104</v>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O22" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P22" s="5" t="n"/>
+      <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t>notebooks/20_interaction_te_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R22" s="4" t="inlineStr">
+        <is>
+          <t>Interaction TE 6쌍 추가: 시술 당시 나이×시술 유형, 시술 당시 나이×특정 시술 유형, 시술 당시 나이×난자 출처, 시술 당시 나이×배란 유도 유형, 시술 유형×총 시술 횟수, 난자 출처×시술 유형</t>
+        </is>
+      </c>
+      <c r="S22" s="4" t="inlineStr">
+        <is>
+          <t>EXP-023 대비 -0.00002 | base LGB=0.74035 CAT=0.74026 XGB=0.74043 | 피처 수 104</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>EXP-025</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>LGB-Optuna-v2(TE)</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>LGB Optuna 50trials | FE-v2+TE(9cols) | lr=0.0137 leaves=126 depth=5</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>0.5175</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>0.78189</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>0.38673</v>
+      </c>
+      <c r="I23" s="8" t="n">
+        <v>0.6233300000000001</v>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>0.74051</v>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L23" s="7" t="inlineStr">
+        <is>
+          <t>v2+TE</t>
+        </is>
+      </c>
+      <c r="M23" s="6" t="n">
+        <v>98</v>
+      </c>
+      <c r="N23" s="7" t="inlineStr">
+        <is>
+          <t>is_unbalance</t>
+        </is>
+      </c>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P23" s="8" t="n"/>
+      <c r="Q23" s="7" t="inlineStr">
+        <is>
+          <t>notebooks/21_hparam_lgb_te_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R23" s="7" t="inlineStr">
+        <is>
+          <t>EXP-019 이후 TE 피처 추가 상태에서 LGB 재튜닝</t>
+        </is>
+      </c>
+      <c r="S23" s="7" t="inlineStr">
+        <is>
+          <t>EXP-019 대비 변화 확인 | 피처 수 98</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>EXP-026</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Ensemble(FE-v2+TE+LGB-v2)</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>FE-v2+TE(9cols) | LGB(EXP-025)+CAT(EXP-011)+XGB(EXP-012) | best=Rank Average</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>0.41062</v>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>0.25835</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>0.25835</v>
+      </c>
+      <c r="J24" s="5" t="n">
+        <v>0.74063</v>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>v2+TE</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O24" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P24" s="5" t="n"/>
+      <c r="Q24" s="4" t="inlineStr">
+        <is>
+          <t>notebooks/22_ensemble_te_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R24" s="4" t="inlineStr">
+        <is>
+          <t>EXP-023 대비 LGB 파라미터를 TE 피처셋 기준 재튜닝(EXP-025)으로 교체</t>
+        </is>
+      </c>
+      <c r="S24" s="4" t="inlineStr">
+        <is>
+          <t>EXP-023 대비 -0.00000 | base LGB=0.74047 CAT=0.74022 XGB=0.74035 | 피처 수 98</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>EXP-027</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Ensemble(LGB+CAT+XGB+MLP)</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>FE-v2+TE | LGB(EXP-025)+CAT(EXP-011)+XGB(EXP-012)+MLP([256-128-64]) | best=Optuna Weights</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>0.5178</v>
+      </c>
+      <c r="G25" s="8" t="n">
+        <v>0.78301</v>
+      </c>
+      <c r="H25" s="8" t="n">
+        <v>0.38679</v>
+      </c>
+      <c r="I25" s="8" t="n">
+        <v>0.62324</v>
+      </c>
+      <c r="J25" s="8" t="n">
+        <v>0.74063</v>
+      </c>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L25" s="7" t="inlineStr">
+        <is>
+          <t>v2+TE</t>
+        </is>
+      </c>
+      <c r="M25" s="6" t="n">
+        <v>98</v>
+      </c>
+      <c r="N25" s="7" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight / oversample(balanced)</t>
+        </is>
+      </c>
+      <c r="O25" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P25" s="8" t="n"/>
+      <c r="Q25" s="7" t="inlineStr">
+        <is>
+          <t>notebooks/23_mlp_ensemble_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R25" s="7" t="inlineStr">
+        <is>
+          <t>MLP(sklearn): [256-128-64] ReLU+Adam lr=0.001 bs=2048 alpha=1e-05</t>
+        </is>
+      </c>
+      <c r="S25" s="7" t="inlineStr">
+        <is>
+          <t>EXP-023 대비 +0.00000 | MLP OOF=0.67588 | Optuna MLP weight=0.006 | 피처 수 98</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>EXP-028</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>SeedEnsemble(LGB+CAT+XGB, 5seeds)</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>EXP-020 파라미터 | seeds=[42, 0, 123, 2024, 777] | best=Optuna Weights</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>0.51795</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>0.78387</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>0.38675</v>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>0.62304</v>
+      </c>
+      <c r="J26" s="5" t="n">
+        <v>0.74082</v>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O26" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="P26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.7421544648	</t>
+        </is>
+      </c>
+      <c r="Q26" s="4" t="inlineStr">
+        <is>
+          <t>notebooks/24_seed_ensemble_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R26" s="4" t="inlineStr">
+        <is>
+          <t>시드 앙상블: 5시드 × 3모델 = 15개 | seeds=[42, 0, 123, 2024, 777]</t>
+        </is>
+      </c>
+      <c r="S26" s="4" t="inlineStr">
+        <is>
+          <t>EXP-020 대비 +0.00014 | LGB=0.74073 CAT=0.74037 XGB=0.74078 | Optuna: LGB=0.347 CAT=0.154 XGB=0.499</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>EXP-029</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Ensemble(LGB+CAT+XGB+TabNet)</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>FE-v1+TabNet(n_d=32,n_steps=3) | LGB(EXP-019)+CAT(EXP-011)+XGB(EXP-012)+TabNet | best=Optuna Weights (4) | LGB=0.303 CAT=0.130 XGB=0.487 Tab=0.080</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>0.51786</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>0.78399</v>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>0.38662</v>
+      </c>
+      <c r="I27" s="8" t="n">
+        <v>0.62286</v>
+      </c>
+      <c r="J27" s="8" t="n">
+        <v>0.7407</v>
+      </c>
+      <c r="K27" s="6" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L27" s="7" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="M27" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="N27" s="7" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight / TabNet weights=1</t>
+        </is>
+      </c>
+      <c r="O27" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P27" s="8" t="n"/>
+      <c r="Q27" s="7" t="inlineStr">
+        <is>
+          <t>notebooks/25_tabnet_ensemble_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R27" s="7" t="inlineStr">
+        <is>
+          <t>TabNet(n_d=32,n_steps=3,gamma=1.3,ep=200,patience=20) + GBDT 3종 앙상블. best=Optuna Weights (4)</t>
+        </is>
+      </c>
+      <c r="S27" s="7" t="inlineStr">
+        <is>
+          <t>EXP-020 대비 +0.00002 | TabNet OOF=0.73347 | LGB=0.74044 CAT=0.74009 XGB=0.74051</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>EXP-031</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Ensemble(LGB-DART+CAT+XGB)</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>LGB(DART,drop=0.1,skip=0.5,rounds=1000)+CAT(EXP-011)+XGB(EXP-012) | best=Optuna Weights | LGB=0.080 CAT=0.269 XGB=0.651</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>0.51781</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>0.78352</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>0.38668</v>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>0.62301</v>
+      </c>
+      <c r="J28" s="5" t="n">
+        <v>0.7406199999999999</v>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O28" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P28" s="5" t="n"/>
+      <c r="Q28" s="4" t="inlineStr">
+        <is>
+          <t>notebooks/27_dart_ensemble_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R28" s="4" t="inlineStr">
+        <is>
+          <t>LGB DART booster(drop_rate=0.1, skip_drop=0.5, rounds=1000). best=Optuna Weights</t>
+        </is>
+      </c>
+      <c r="S28" s="4" t="inlineStr">
+        <is>
+          <t>EXP-020 대비 -0.00006 | LGB(DART)=0.73980 CAT=0.74015 XGB=0.74051 | EXP-020 LGB(GBDT)=0.74047</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>EXP-032</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Ensemble(LGB-v1+CAT-TE+XGB-ITE)</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>LGB(FE-v1,85f)+CAT(FE-v2+TE,98f)+XGB(FE-v2+TE+ITE,104f) | best=Rank Average | LGB=0.417 CAT=0.275 XGB=0.308</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="n">
+        <v>0.41062</v>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" s="8" t="n">
+        <v>0.25835</v>
+      </c>
+      <c r="I29" s="8" t="n">
+        <v>0.25835</v>
+      </c>
+      <c r="J29" s="8" t="n">
+        <v>0.74071</v>
+      </c>
+      <c r="K29" s="6" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>mixed(v1/v2/TE/ITE)</t>
+        </is>
+      </c>
+      <c r="M29" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="N29" s="7" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O29" s="6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="P29" s="8" t="inlineStr">
+        <is>
+          <t>0.742192764</t>
+        </is>
+      </c>
+      <c r="Q29" s="7" t="inlineStr">
+        <is>
+          <t>notebooks/28_mixed_fe_ensemble_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R29" s="7" t="inlineStr">
+        <is>
+          <t>모델별 다른 피처셋: LGB=FE-v1, CAT=FE-v2+TE, XGB=FE-v2+TE+ITE. 예측 다양성 확보 목적</t>
+        </is>
+      </c>
+      <c r="S29" s="7" t="inlineStr">
+        <is>
+          <t>EXP-020 대비 +0.00003 | LGB(v1)=0.74047 CAT(v2+TE)=0.74022 XGB(v2+TE+ITE)=0.74043</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>EXP-033</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Super-Ensemble(RankAvg)</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>RankAvg(EXP-020+EXP-028+EXP-031+EXP-032) | 새 학습 없음, 기존 test 예측 앙상블</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
+      <c r="H30" s="5" t="n"/>
+      <c r="I30" s="5" t="n"/>
+      <c r="J30" s="5" t="n">
+        <v>0.74071</v>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>N/A (test-only)</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="n"/>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="O30" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P30" s="5" t="n"/>
+      <c r="Q30" s="4" t="inlineStr">
+        <is>
+          <t>notebooks/29_super_ensemble_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R30" s="4" t="inlineStr">
+        <is>
+          <t>Super-ensemble: 기존 4개 실험 test 예측 Rank Average. OOF AUC는 소스 실험 평균값(proxy). 주의: EXP-020≈EXP-032(corr=0.9996), EXP-028≈EXP-031(corr=0.9999) — 실질적 2그룹 앙상블.</t>
+        </is>
+      </c>
+      <c r="S30" s="4" t="inlineStr">
+        <is>
+          <t>EXP-020(0.74217)+EXP-028(0.74215)+EXP-031(미제출)+EXP-032(0.74219) rank avg | 가장 다양한 조합: EXP-028+EXP-032(corr=0.9609) | 3개 조합 비교용 파일도 저장됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>EXP-034</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Unified(EXP-020+028+032)</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>RankAvg(EXP-020+EXP-028+EXP-032) | A:LGB+CAT+XGB(seed=42,FE-v1) + B:LGB+CAT+XGB(5seeds,FE-v1) + C:LGB(FE-v1)+CAT(FE-v2+TE)+XGB(FE-v2+TE+ITE)</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="n">
+        <v>0.51733</v>
+      </c>
+      <c r="G31" s="8" t="n">
+        <v>0.75997</v>
+      </c>
+      <c r="H31" s="8" t="n">
+        <v>0.39213</v>
+      </c>
+      <c r="I31" s="8" t="n">
+        <v>0.63364</v>
+      </c>
+      <c r="J31" s="8" t="n">
+        <v>0.74081</v>
+      </c>
+      <c r="K31" s="6" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L31" s="7" t="inlineStr">
+        <is>
+          <t>mixed(v1/v2/TE/ITE)</t>
+        </is>
+      </c>
+      <c r="M31" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="N31" s="7" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O31" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P31" s="8" t="n"/>
+      <c r="Q31" s="7" t="inlineStr">
+        <is>
+          <t>notebooks/30_final_code_submission_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R31" s="7" t="inlineStr">
+        <is>
+          <t>대회 코드 제출용 통합 노트북. EXP-020+028+032 파이프라인 통합 + Rank Average 최종 앙상블.</t>
+        </is>
+      </c>
+      <c r="S31" s="7" t="inlineStr">
+        <is>
+          <t>A(EXP-020)=0.74068  B(EXP-028)=0.74081  C(EXP-032)=0.74071  Final=0.74081</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>EXP-035</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>RF+ET Ensemble</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>RF(n=500,leaf=20,balanced)+ET(n=500,leaf=20,balanced) | 앙상블: RF+ET+EXP-020+EXP-028+EXP-032 Rank Avg</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>0.5141</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>0.7440099999999999</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>0.39273</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>0.63665</v>
+      </c>
+      <c r="J32" s="5" t="n">
+        <v>0.73631</v>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>class_weight=balanced</t>
+        </is>
+      </c>
+      <c r="O32" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P32" s="5" t="n"/>
+      <c r="Q32" s="4" t="inlineStr">
+        <is>
+          <t>notebooks/31_rf_ensemble_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R32" s="4" t="inlineStr">
+        <is>
+          <t>RF/ET 단독 OOF AUC 기록. 앙상블은 기존 submission 파일과 test 예측 결합. RF ↔ GBDT 상관관계 낮으면 앙상블 효과 큼.</t>
+        </is>
+      </c>
+      <c r="S32" s="4" t="inlineStr">
+        <is>
+          <t>RF=0.73631  ET=0.73575  RF+ET=0.73672 | GBDT 기준선 0.74068 대비 -0.00437 (RF 단독)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>EXP-036</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Ensemble(LGB-DART-TE+CAT-TE+XGB-ITE)</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>LGB(DART,drop=0.1,rounds=1000,FE-v2+TE,98f)+CAT(FE-v2+TE,98f)+XGB(FE-v2+TE+ITE,104f) | best=Optuna Weights | LGB=0.106 CAT=0.350 XGB=0.544</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="n">
+        <v>0.5181</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>0.78492</v>
+      </c>
+      <c r="H33" s="8" t="n">
+        <v>0.38666</v>
+      </c>
+      <c r="I33" s="8" t="n">
+        <v>0.62276</v>
+      </c>
+      <c r="J33" s="8" t="n">
+        <v>0.7406</v>
+      </c>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L33" s="7" t="inlineStr">
+        <is>
+          <t>v2+TE+ITE</t>
+        </is>
+      </c>
+      <c r="M33" s="6" t="n">
+        <v>89</v>
+      </c>
+      <c r="N33" s="7" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O33" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P33" s="8" t="n"/>
+      <c r="Q33" s="7" t="inlineStr">
+        <is>
+          <t>notebooks/32_dart_te_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R33" s="7" t="inlineStr">
+        <is>
+          <t>EXP-031(DART)+EXP-032(TE) 조합. LGB에만 DART 적용, CAT/XGB는 EXP-032 동일.</t>
+        </is>
+      </c>
+      <c r="S33" s="7" t="inlineStr">
+        <is>
+          <t>EXP-032 대비 -0.00011 | LGB(DART+TE)=0.73986 CAT(TE)=0.74022 XGB(TE+ITE)=0.74043</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>EXP-037</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Stacking(LGB+CAT+XGB ×2 → LGB-meta)</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>L1: LGB+CAT+XGB(FE-v1) + LGB+CAT+XGB(FE-v2+TE+ITE) | L2: LGB(leaves=8,depth=3) | best=Rank Average</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>0.51759</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>0.78239</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>0.38671</v>
+      </c>
+      <c r="I34" s="5" t="n">
+        <v>0.62322</v>
+      </c>
+      <c r="J34" s="5" t="n">
+        <v>0.74073</v>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>mixed(v1/v2+TE+ITE)</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O34" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P34" s="5" t="n"/>
+      <c r="Q34" s="4" t="inlineStr">
+        <is>
+          <t>notebooks/33_stacking_v2_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R34" s="4" t="inlineStr">
+        <is>
+          <t>Stacking: 6개 Base 모델 OOF → LGB Meta 학습. FE-v1 3개 + FE-v2+TE+ITE 3개. Meta LGB는 과적합 방지 위해 shallow (leaves=8, depth=3).</t>
+        </is>
+      </c>
+      <c r="S34" s="4" t="inlineStr">
+        <is>
+          <t>EXP-032 대비 +0.00002 | Stacking=0.74002 vs RankAvg(6모델)=0.74073 | Stacking 개선: -0.00071</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>EXP-038</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>MultiSeed-EXP032(LGB+CAT+XGB×5seeds)</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>MultiSeed(5) × EXP-032 | seeds=[42, 0, 123, 2024, 777] | LGB(FE-v1)+CAT(FE-v2+TE)+XGB(FE-v2+TE+ITE) per seed | 15모델 RankAvg</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="n">
+        <v>0.5175999999999999</v>
+      </c>
+      <c r="G35" s="8" t="n">
+        <v>0.76066</v>
+      </c>
+      <c r="H35" s="8" t="n">
+        <v>0.39226</v>
+      </c>
+      <c r="I35" s="8" t="n">
+        <v>0.6337</v>
+      </c>
+      <c r="J35" s="8" t="n">
+        <v>0.7409</v>
+      </c>
+      <c r="K35" s="6" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold × 5 seeds</t>
+        </is>
+      </c>
+      <c r="L35" s="7" t="inlineStr">
+        <is>
+          <t>mixed(v1/v2+TE+ITE)</t>
+        </is>
+      </c>
+      <c r="M35" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="N35" s="7" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O35" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P35" s="8" t="n"/>
+      <c r="Q35" s="7" t="inlineStr">
+        <is>
+          <t>notebooks/34_multi_seed_exp032_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R35" s="7" t="inlineStr">
+        <is>
+          <t>EXP-032 아키텍처(LGB FE-v1 / CAT FE-v2+TE / XGB FE-v2+TE+ITE)를 5개 시드로 반복 학습 후 15개 예측을 Rank Average. TE/ITE는 fold 내부 계산 (data leakage 없음).</t>
+        </is>
+      </c>
+      <c r="S35" s="7" t="inlineStr">
+        <is>
+          <t>EXP-032(seed=42) OOF=0.74071 대비 +0.00019 | EXP-034 OOF=0.74081 대비 +0.00009 | 15모델(5seeds×3models) RankAvg</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>EXP-039</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>4Model-MultiSeed(LGB×2+CAT+XGB×5seeds)</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>MultiSeed(5) × 4모델 | seeds=[42, 0, 123, 2024, 777] | LGB(FE-v1)+CAT(FE-v2+TE)+XGB(FE-v2+TE+ITE)+LGB(FE-v2+TE+ITE) | 20모델 RankAvg</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>0.5177</v>
+      </c>
+      <c r="G36" s="5" t="n">
+        <v>0.76083</v>
+      </c>
+      <c r="H36" s="5" t="n">
+        <v>0.39233</v>
+      </c>
+      <c r="I36" s="5" t="n">
+        <v>0.6337699999999999</v>
+      </c>
+      <c r="J36" s="5" t="n">
+        <v>0.74091</v>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold × 5 seeds</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>mixed(v1/v2+TE+ITE)</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O36" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P36" s="5" t="n"/>
+      <c r="Q36" s="4" t="inlineStr">
+        <is>
+          <t>notebooks/35_multi_seed_4model_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R36" s="4" t="inlineStr">
+        <is>
+          <t>EXP-038(15모델)에 LGB(FE-v2+TE+ITE) 추가 → 20모델 Rank Average. XGB와 동일 피처에 LGB 사용으로 알고리즘 다양성 확보. TE/ITE는 fold 내부 계산 (data leakage 없음).</t>
+        </is>
+      </c>
+      <c r="S36" s="4" t="inlineStr">
+        <is>
+          <t>EXP-038 OOF=0.74090 대비 +0.00001 | EXP-032 제출 0.74219 대비 | 20모델(5seeds×4models) RankAvg</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>EXP-040</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>MultiSeed10-EXP032(LGB+CAT+XGB×10seeds)</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>MultiSeed(10) × EXP-032 아키텍처 | seeds=[42, 0, 123, 2024, 777, 1, 99, 314, 2023, 500] | LGB(FE-v1)+CAT(FE-v2+TE)+XGB(FE-v2+TE+ITE) | 30모델 RankAvg</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="n">
+        <v>0.51774</v>
+      </c>
+      <c r="G37" s="8" t="n">
+        <v>0.76068</v>
+      </c>
+      <c r="H37" s="8" t="n">
+        <v>0.39241</v>
+      </c>
+      <c r="I37" s="8" t="n">
+        <v>0.63389</v>
+      </c>
+      <c r="J37" s="8" t="n">
+        <v>0.74091</v>
+      </c>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold × 10 seeds</t>
+        </is>
+      </c>
+      <c r="L37" s="7" t="inlineStr">
+        <is>
+          <t>mixed(v1/v2+TE+ITE)</t>
+        </is>
+      </c>
+      <c r="M37" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="N37" s="7" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O37" s="6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P37" s="8" t="n">
+        <v>0.7422343142</v>
+      </c>
+      <c r="Q37" s="7" t="inlineStr">
+        <is>
+          <t>notebooks/36_multi_seed_10s_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R37" s="7" t="inlineStr">
+        <is>
+          <t>EXP-038(5seeds→30모델)의 씨드 확장 버전. 10 seeds × 3 models = 30모델 Rank Average. TE/ITE는 fold 내부 계산 (data leakage 없음).</t>
+        </is>
+      </c>
+      <c r="S37" s="7" t="inlineStr">
+        <is>
+          <t>EXP-038(5seeds) OOF=0.74090 대비 +0.00001 | 예상 제출 점수: 0.74239 | 1등(0.74246) 기준: 미달 | 최종 리더보드 4위 (1위:0.74246, 2위:0.74237, 3위:0.74228, 4위:0.74223)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>EXP-041</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>조여진</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>CAT-ITE+ITE10+MultiSeed5(LGB+CAT×2+XGB)</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>MultiSeed(5) × 4모델 | ITE 6→10쌍 확장 | seeds=[42, 0, 123, 2024, 777] | LGB(FE-v1)+CAT(TE)+CAT(TE+ITE_10)+XGB(TE+ITE_10) | 20모델 RankAvg</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>0.51771</v>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>0.76052</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <v>0.39242</v>
+      </c>
+      <c r="I38" s="5" t="n">
+        <v>0.63393</v>
+      </c>
+      <c r="J38" s="5" t="n">
+        <v>0.74086</v>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Stratified 5-Fold × 5 seeds</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>mixed(v1/v2+TE+ITE10)</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>is_unbalance / Balanced / scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="O38" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P38" s="5" t="n"/>
+      <c r="Q38" s="4" t="inlineStr">
+        <is>
+          <t>notebooks/37_cat_ite_expanded_yjcho.ipynb</t>
+        </is>
+      </c>
+      <c r="R38" s="4" t="inlineStr">
+        <is>
+          <t>CAT에 ITE 첫 적용. ITE 6쌍→10쌍 확장(신규: 나이×총임신횟수, 나이×총시술횟수, 배란유도유형×난자출처, 특정시술유형×난자출처). 4모델(LGB-v1+CAT-TE+CAT-ITE10+XGB-ITE10)×5seeds=20모델 RankAvg.</t>
+        </is>
+      </c>
+      <c r="S38" s="4" t="inlineStr">
+        <is>
+          <t>EXP-038(5seeds 3models) OOF=0.74090 대비 -0.00004 | CAT2(ITE) 기여: -0.00003 | 예상 제출: 0.74234</t>
         </is>
       </c>
     </row>

</xml_diff>